<commit_message>
Flor de lis, Viagem a Santiago, quotas de secção e versão de telemóvel
- Categorias: 'Quotas de secção' nas entradas; sai 'Quotas nacionais e seguros'
- Meta de exemplo passa a ser a Viagem a Santiago
- Flor de lis no título e no ícone do separador
- Telemóvel: sem scroll lateral, gráfico mês a mês ajusta-se ao ecrã e
  responde ao toque, movimentos em cartões
- Site marcado para não aparecer em motores de busca

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Folha-Tesouraria-Exploradores.xlsx
+++ b/Folha-Tesouraria-Exploradores.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Quotas dos exploradores</t>
+          <t>Quotas de secção</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Quotas nacionais e seguros</t>
+          <t>Material e equipamento</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -533,11 +533,11 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>768</v>
+        <v>224.9</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Fatura nº 2026-114</t>
+          <t>Talão Decathlon 27/09</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       <formula1>"Entrada,Saída"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Categorias!$B$2:$B$13</formula1>
+      <formula1>=Categorias!$B$2:$B$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4609,14 +4609,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Acampamento de verão 2027</t>
+          <t>Viagem a Santiago</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46569</v>
+        <v>46583</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -4724,11 +4724,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Quotas nacionais e seguros</t>
+          <t>Insígnias e cerimónias</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>800</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7">
@@ -4739,27 +4739,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Insígnias e cerimónias</t>
+          <t>Outras despesas</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>250</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>2026/27</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Outras despesas</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>400</v>
-      </c>
+      <c r="A8" s="4" t="n"/>
+      <c r="C8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
@@ -5528,7 +5517,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Categorias!$B$2:$B$8</formula1>
+      <formula1>=Categorias!$B$2:$B$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5541,7 +5530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5616,7 +5605,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Quotas nacionais e seguros</t>
+          <t>Insígnias e cerimónias</t>
         </is>
       </c>
     </row>
@@ -5628,19 +5617,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Insígnias e cerimónias</t>
+          <t>Outras despesas</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Outras despesas</t>
+          <t>Quotas de secção</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5641,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Quotas dos exploradores</t>
+          <t>Angariação de fundos</t>
         </is>
       </c>
     </row>
@@ -5664,7 +5653,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Angariação de fundos</t>
+          <t>Subsídio do agrupamento</t>
         </is>
       </c>
     </row>
@@ -5676,7 +5665,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Subsídio do agrupamento</t>
+          <t>Donativos</t>
         </is>
       </c>
     </row>
@@ -5687,18 +5676,6 @@
         </is>
       </c>
       <c r="B12" t="inlineStr">
-        <is>
-          <t>Donativos</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Entrada</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
         <is>
           <t>Outras entradas</t>
         </is>

</xml_diff>

<commit_message>
Secção Caminho de Santiago 2027
- Fundo da viagem (entradas com 'Santiago' na atividade), o que falta,
  por participante e por mês, contagem decrescente
- Orçamento previsto por rubrica (voos, alimentação, dormidas, transporte
  local, margem), três cenários de custo e itinerário dia a dia
- Painel 'Por atividade' com o resultado de cada atividade do ano
- O Gemini conhece o plano da viagem; folha modelo com a meta de 6'000

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Folha-Tesouraria-Exploradores.xlsx
+++ b/Folha-Tesouraria-Exploradores.xlsx
@@ -4609,14 +4609,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Viagem a Santiago</t>
+          <t>Caminho de Santiago 2027</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>9000</v>
+        <v>6000</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46583</v>
+        <v>46638</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>

</xml_diff>